<commit_message>
vault backup: 2026-06-04 21:07:54
</commit_message>
<xml_diff>
--- a/roofing-target-list.xlsx
+++ b/roofing-target-list.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -45,6 +45,11 @@
     <font>
       <name val="Arial"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <i val="1"/>
+      <color rgb="007F7F7F"/>
     </font>
   </fonts>
   <fills count="9">
@@ -116,7 +121,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -152,6 +157,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -517,7 +523,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J34"/>
+  <dimension ref="A1:J55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -2089,6 +2095,933 @@
           <t>5/31/2026</t>
         </is>
       </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="13" t="inlineStr">
+        <is>
+          <t>--- BATCH 2 (appended 6/3/2026 via web search — verify connection degree on LinkedIn before sending) ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>31</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Ron Osbon</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Rao Roofing</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Grant, MI</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Unknown — verify (re-find attempt: found)</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Good — verify size | RE-FOUND from Batch 1 skip</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Ron — fellow roofing operator here. Always glad to connect with owners running real crews in Michigan. Would be good to be connected.</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Pending — Batch 2</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>32</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Jack Petsche</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>USA Roofing Inc.</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Twinsburg, OH</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Unknown — verify</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Good — 30+ yr operator, verify size</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Jack — roofing operator here. 30 years in the trade commands respect. Always up for connecting with owners running real shops in Ohio. Connect?</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Pending — Batch 2</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>33</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>John Andres</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Andres Roofing Co.</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Florida (verify city)</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Unknown — verify</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Good — verify size</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>John — fellow roofing operator. Like connecting with owners who've built something real in FL. Would be good to be connected.</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Pending — Batch 2</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>34</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>David Crowther</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>President</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>CFS Roofing Services LLC</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Fort Myers, FL</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Unknown — verify</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Good — res/commercial, verify size</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>David — roofing operator here too. Like connecting with owners running solid commercial/res shops in SW Florida. Connect?</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Pending — Batch 2</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>35</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Matt O'Rear</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Apex Roofing of Coastal Georgia LLC</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Savannah/Brunswick area, GA</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Unknown — verify</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Good — coastal storm market, verify size</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Matt — fellow roofing operator. Coastal GA is a solid storm market. Like connecting with owners building real crews there. Connect?</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Pending — Batch 2</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>36</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Nicholas Hildom</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Texas Roofing Authority</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Austin, TX</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Unknown — verify</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Good — verify size, Austin TX</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Nicholas — roofing operator here too. Like connecting with owners running real crews in the Austin market. Open to connecting?</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Pending — Batch 2</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>37</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Jason Wendlandt</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Minnesota Roofing Contractors LLC</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Belle Plaine, MN</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Unknown — verify</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Good — verify size</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Jason — fellow roofing operator in the Upper Midwest. Like connecting with owners running real shops in MN. Would be good to connect.</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Pending — Batch 2</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>38</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Raymond Byrne</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>President</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>America Roofing LLC</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Phoenix, AZ</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Unknown — verify</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Good — verify size, Phoenix</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Raymond — roofing operator here too. The Phoenix market is no joke for volume. Like connecting with owners running real teams there. Connect?</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Pending — Batch 2</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>39</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Don Harrelson</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Best Roofing of Virginia</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Virginia Beach, VA</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Unknown — verify</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Good — verify size, Hampton Roads</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Don — fellow roofing operator. Like connecting with owners running solid shops in the Hampton Roads market. Would be good to connect.</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Pending — Batch 2</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>40</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Thomas Hennessey</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Owner-President</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Hennessey Roofing, LLC</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>United States (verify)</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Unknown — verify</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Good — verify size &amp; location</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Thomas — fellow roofing operator. Always glad to connect with owners who built their own shop. Would be good to be connected.</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Pending — Batch 2</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>41</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Kevin Sweeney</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Advanced Roofing and Exteriors</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>United States (verify state)</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Unknown — verify</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Good — res/exteriors, verify size &amp; location</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Kevin — roofing/exteriors operator here too. Like connecting with owners running real crews on the res side. Open to connecting?</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Pending — Batch 2</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>42</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>David Rosato</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>5 Stars Roofing LLC</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Charleston, SC area</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Unknown — verify</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Good — verify size, coastal SC</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>David — fellow roofing operator. Like connecting with owners building real crews in the Carolinas coastal market. Would be good to connect.</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Pending — Batch 2</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>43</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Walter Murphy</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Pro Com Roofing Corp.</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Warrington, PA</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Unknown — verify</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Good — verify size</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Walter — roofing operator here. Like connecting with owners running real commercial/res crews in PA. Would be good to be connected.</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Pending — Batch 2</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>44</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Nathan Sockman</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Owner/Principal</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Meade Roofing Services, Inc.</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Pennsylvania</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Unknown — verify</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Good — verify size &amp; exact title</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Nathan — fellow roofing operator. Always glad to connect with owners running solid shops in PA. Would be good to be connected.</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Pending — Batch 2</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>45</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Gary Sova</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>President</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>National Roofing &amp; Sheet Metal Co Inc</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Burton, MI</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Unknown — verify</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Partial — commercial/sheet metal focus, verify size</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Gary — roofing/sheet metal operator here too. Like connecting with operators who roll their own metal in Michigan. Connect?</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Pending — Batch 2</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>46</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Dennis Boothe</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>President/Owner</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Roof-Pro, Inc.</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>United States (verify state)</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Unknown — verify</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Good — 35 yr commercial/industrial, verify size</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Dennis — 35 years in commercial/industrial roofing is serious time. Fellow operator. Always glad to connect with owners who've built it. Connect?</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Pending — Batch 2</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>47</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Eric Taylor</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Elite Roofing LLC</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>United States (verify)</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Unknown — verify</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Good — verify size &amp; location</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Eric — fellow roofing operator. Like connecting with owners running real crews. Would be good to be connected.</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Pending — Batch 2</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>48</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Jason Milliken</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>VP/General Manager</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Texas Roofing Co.</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Elgin, TX</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Unknown — verify</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Partial — VP/GM not owner; verify co. size &amp; owner relationship</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Jason — fellow roofing operator, I know the TX market. Like connecting with GMs/VPs running real ops in the Dallas-Austin corridor. Connect?</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Pending — Batch 2</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>49</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Zac Ammons</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Core Commercial Roofing &amp; Liquid Seal</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>United States (verify)</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Unknown — verify</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Partial — commercial focus; verify size</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Zac — commercial roofer here too. Like connecting with owners/operators running real commercial crews. Would be good to be connected.</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Pending — Batch 2</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>50</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Martin Cromer</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Owner/President</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>M C Roofing Enterprises LLC</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>United States (verify)</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Unknown — verify</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Good — verify size &amp; location</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Martin — fellow roofing operator. Like connecting with owners who built something real. Would be good to be connected.</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Pending — Batch 2</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>